<commit_message>
Use FALTANTE vs inventario instead of FALTANTE PRIORITARIO
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MOTION_LOOP_PRIORITARIO_REAL.xlsx
+++ b/MOTION_LOOP_PRIORITARIO_REAL.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prioritario Real" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Solo Prioritario Real" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Faltante Real" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Solo Faltante Real" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Cubierto por Inventario" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Inventario sin Faltante" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,22 +462,17 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>FALTANTE PRIORITARIO</t>
+          <t>INVENTARIO MANUFACTURA</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>INVENTARIO MANUFACTURA</t>
+          <t>CUBIERTO POR INVENTARIO</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>CUBIERTO POR INVENTARIO</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>PRIORITARIO REAL</t>
+          <t>FALTANTE REAL</t>
         </is>
       </c>
     </row>
@@ -517,17 +512,14 @@
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -563,15 +555,12 @@
         <v>40</v>
       </c>
       <c r="I3" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="J3" t="n">
         <v>23</v>
       </c>
       <c r="K3" t="n">
-        <v>23</v>
-      </c>
-      <c r="L3" t="n">
         <v>17</v>
       </c>
     </row>
@@ -609,16 +598,13 @@
         <v>40</v>
       </c>
       <c r="I4" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="J4" t="n">
         <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L4" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -657,16 +643,13 @@
         <v>10</v>
       </c>
       <c r="I5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J5" t="n">
         <v>4</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -703,16 +686,13 @@
         <v>40</v>
       </c>
       <c r="I6" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="J6" t="n">
         <v>8</v>
       </c>
       <c r="K6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L6" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -757,9 +737,6 @@
         <v>6</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
-      </c>
-      <c r="L7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -797,15 +774,12 @@
         <v>24</v>
       </c>
       <c r="I8" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
         <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" t="n">
         <v>22</v>
       </c>
     </row>
@@ -851,10 +825,7 @@
         <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -893,17 +864,14 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
+        <v>8</v>
+      </c>
+      <c r="J10" t="n">
         <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>8</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -941,15 +909,12 @@
         <v>15</v>
       </c>
       <c r="I11" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="J11" t="n">
         <v>7</v>
       </c>
       <c r="K11" t="n">
-        <v>7</v>
-      </c>
-      <c r="L11" t="n">
         <v>8</v>
       </c>
     </row>
@@ -989,17 +954,14 @@
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1035,16 +997,13 @@
         <v>24</v>
       </c>
       <c r="I13" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
         <v>4</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -1083,17 +1042,14 @@
         <v>5</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J14" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1131,17 +1087,14 @@
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="J15" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1179,17 +1132,14 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" t="n">
         <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>4</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1225,15 +1175,12 @@
         <v>40</v>
       </c>
       <c r="I17" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="J17" t="n">
         <v>8</v>
       </c>
       <c r="K17" t="n">
-        <v>8</v>
-      </c>
-      <c r="L17" t="n">
         <v>32</v>
       </c>
     </row>
@@ -1271,16 +1218,13 @@
         <v>24</v>
       </c>
       <c r="I18" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="J18" t="n">
         <v>3</v>
       </c>
       <c r="K18" t="n">
-        <v>3</v>
-      </c>
-      <c r="L18" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19">
@@ -1319,7 +1263,7 @@
         <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
@@ -1327,9 +1271,6 @@
       <c r="K19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1367,17 +1308,14 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1413,16 +1351,13 @@
         <v>40</v>
       </c>
       <c r="I21" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="J21" t="n">
         <v>8</v>
       </c>
       <c r="K21" t="n">
-        <v>8</v>
-      </c>
-      <c r="L21" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22">
@@ -1461,15 +1396,12 @@
         <v>2</v>
       </c>
       <c r="I22" t="n">
+        <v>48</v>
+      </c>
+      <c r="J22" t="n">
         <v>2</v>
       </c>
-      <c r="J22" t="n">
-        <v>48</v>
-      </c>
       <c r="K22" t="n">
-        <v>2</v>
-      </c>
-      <c r="L22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1507,16 +1439,13 @@
         <v>24</v>
       </c>
       <c r="I23" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="J23" t="n">
         <v>4</v>
       </c>
       <c r="K23" t="n">
-        <v>4</v>
-      </c>
-      <c r="L23" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24">
@@ -1553,15 +1482,12 @@
         <v>16</v>
       </c>
       <c r="I24" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1601,17 +1527,14 @@
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J25" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1649,16 +1572,13 @@
         <v>26</v>
       </c>
       <c r="I26" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J26" t="n">
         <v>24</v>
       </c>
       <c r="K26" t="n">
-        <v>16</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -1697,7 +1617,7 @@
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J27" t="n">
         <v>1</v>
@@ -1705,9 +1625,6 @@
       <c r="K27" t="n">
         <v>1</v>
       </c>
-      <c r="L27" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1745,17 +1662,14 @@
         <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J28" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1793,17 +1707,14 @@
         <v>4</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="J29" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
       </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1841,15 +1752,12 @@
         <v>13</v>
       </c>
       <c r="I30" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="J30" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
-      </c>
-      <c r="L30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1889,15 +1797,12 @@
         <v>4</v>
       </c>
       <c r="I31" t="n">
+        <v>32</v>
+      </c>
+      <c r="J31" t="n">
         <v>4</v>
       </c>
-      <c r="J31" t="n">
-        <v>32</v>
-      </c>
       <c r="K31" t="n">
-        <v>4</v>
-      </c>
-      <c r="L31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1935,15 +1840,12 @@
         <v>24</v>
       </c>
       <c r="I32" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="J32" t="n">
         <v>4</v>
       </c>
       <c r="K32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L32" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1981,15 +1883,12 @@
         <v>16</v>
       </c>
       <c r="I33" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2029,15 +1928,12 @@
         <v>7</v>
       </c>
       <c r="I34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J34" t="n">
         <v>6</v>
       </c>
       <c r="K34" t="n">
-        <v>6</v>
-      </c>
-      <c r="L34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2075,15 +1971,12 @@
         <v>24</v>
       </c>
       <c r="I35" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="J35" t="n">
         <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>2</v>
-      </c>
-      <c r="L35" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2123,15 +2016,12 @@
         <v>3</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J36" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2146,7 +2036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2192,39 +2082,34 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>FALTANTE PRIORITARIO</t>
+          <t>INVENTARIO MANUFACTURA</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>INVENTARIO MANUFACTURA</t>
+          <t>CUBIERTO POR INVENTARIO</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>CUBIERTO POR INVENTARIO</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>PRIORITARIO REAL</t>
+          <t>FALTANTE REAL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MLMMJDA12TM</t>
+          <t>MLCMJCA12TS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MOTION LOOP MAFE</t>
+          <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2234,7 +2119,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -2245,68 +2130,62 @@
         <v>40</v>
       </c>
       <c r="I2" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
         <v>8</v>
       </c>
       <c r="K2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L2" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MLCMJCA14TL</t>
+          <t>MLMMJDA12TM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MOTION LOOP CLASICA</t>
+          <t>MOTION LOOP MAFE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CAB</t>
+          <t>DAMA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Azul Turquesa</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="I3" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L3" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MLCMJCA12TS</t>
+          <t>MLCMJCA14TS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2321,7 +2200,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Azul Marino</t>
+          <t>Azul Turquesa</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2337,32 +2216,29 @@
         <v>40</v>
       </c>
       <c r="I4" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="J4" t="n">
         <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L4" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MLCMJCA50TL</t>
+          <t>MLMMJDA50TS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MOTION LOOP CLASICA</t>
+          <t>MOTION LOOP MAFE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CAB</t>
+          <t>DAMA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2372,33 +2248,30 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="I5" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L5" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MLCMJCA14TS</t>
+          <t>MLCMJCA50TL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2413,84 +2286,78 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Azul Turquesa</t>
+          <t>Rojo</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="I6" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L6" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MLMMJDA50TS</t>
+          <t>MLCMJCA14TL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MOTION LOOP MAFE</t>
+          <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Azul Turquesa</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="I7" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MLMMJDA14TL</t>
+          <t>MLMMJDA12TL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2505,7 +2372,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Azul Turquesa</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2521,88 +2388,82 @@
         <v>24</v>
       </c>
       <c r="I8" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>4</v>
-      </c>
-      <c r="L8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MLCMJCA12TM</t>
+          <t>MLMMJDA14TL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MOTION LOOP CLASICA</t>
+          <t>MOTION LOOP MAFE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CAB</t>
+          <t>DAMA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Azul Marino</t>
+          <t>Azul Turquesa</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="I9" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="J9" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
-        <v>23</v>
-      </c>
-      <c r="L9" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MLMMJDA12TL</t>
+          <t>MLCMJCA66TXL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MOTION LOOP MAFE</t>
+          <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Azul Marino</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -2613,22 +2474,19 @@
         <v>24</v>
       </c>
       <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" t="n">
         <v>20</v>
-      </c>
-      <c r="J10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MLMMJDA14TXL</t>
+          <t>MLMMJDA50TL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2643,99 +2501,93 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Azul Turquesa</t>
+          <t>Rojo</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I11" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MLMMJDA50TL</t>
+          <t>MLCMJCA12TM</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MOTION LOOP MAFE</t>
+          <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="I12" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
-      </c>
-      <c r="L12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MLCMJCA66TXL</t>
+          <t>MLMMJDA14TXL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MOTION LOOP CLASICA</t>
+          <t>MOTION LOOP MAFE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CAB</t>
+          <t>DAMA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Verde Militar</t>
+          <t>Azul Turquesa</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2744,22 +2596,19 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="I13" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2797,15 +2646,12 @@
         <v>16</v>
       </c>
       <c r="I14" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
-      </c>
-      <c r="L14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2845,15 +2691,12 @@
         <v>15</v>
       </c>
       <c r="I15" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="J15" t="n">
         <v>7</v>
       </c>
       <c r="K15" t="n">
-        <v>7</v>
-      </c>
-      <c r="L15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2893,111 +2736,192 @@
         <v>10</v>
       </c>
       <c r="I16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J16" t="n">
         <v>4</v>
       </c>
       <c r="K16" t="n">
-        <v>4</v>
-      </c>
-      <c r="L16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MLMMJDA66TM</t>
+          <t>MLCMJCA50TXL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MOTION LOOP MAFE</t>
+          <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Verde Militar</t>
+          <t>Rojo</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G17" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>MLMMJDA66TS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>40</v>
+      </c>
+      <c r="G18" t="n">
+        <v>14</v>
+      </c>
+      <c r="H18" t="n">
+        <v>26</v>
+      </c>
+      <c r="I18" t="n">
+        <v>24</v>
+      </c>
+      <c r="J18" t="n">
+        <v>24</v>
+      </c>
+      <c r="K18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MLMMJDA66TM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>40</v>
+      </c>
+      <c r="G19" t="n">
+        <v>38</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>MLCMJCA14TM</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>CAB</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Azul Turquesa</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>40</v>
-      </c>
-      <c r="G18" t="n">
+      <c r="F20" t="n">
+        <v>40</v>
+      </c>
+      <c r="G20" t="n">
         <v>33</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H20" t="n">
         <v>7</v>
       </c>
-      <c r="I18" t="n">
-        <v>7</v>
-      </c>
-      <c r="J18" t="n">
+      <c r="I20" t="n">
         <v>6</v>
       </c>
-      <c r="K18" t="n">
+      <c r="J20" t="n">
         <v>6</v>
       </c>
-      <c r="L18" t="n">
+      <c r="K20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3012,7 +2936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3058,29 +2982,24 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>FALTANTE PRIORITARIO</t>
+          <t>INVENTARIO MANUFACTURA</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>INVENTARIO MANUFACTURA</t>
+          <t>CUBIERTO POR INVENTARIO</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>CUBIERTO POR INVENTARIO</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>PRIORITARIO REAL</t>
+          <t>FALTANTE REAL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MLCMJCA50TM</t>
+          <t>MLCMJCA12TL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3095,40 +3014,37 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G2" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
-      </c>
-      <c r="L2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MLCMJCA50TXL</t>
+          <t>MLCMJCA50TM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3148,93 +3064,87 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G3" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="H3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
-      </c>
-      <c r="L3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MLMMJDA50TM</t>
+          <t>MLCMJCA66TL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MOTION LOOP MAFE</t>
+          <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G4" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="H4" t="n">
         <v>2</v>
       </c>
       <c r="I4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" t="n">
         <v>2</v>
       </c>
-      <c r="J4" t="n">
-        <v>48</v>
-      </c>
       <c r="K4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MLMMJDA66TS</t>
+          <t>MLCMJCA66TS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MOTION LOOP MAFE</t>
+          <t>MOTION LOOP CLASICA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3251,28 +3161,25 @@
         <v>40</v>
       </c>
       <c r="G5" t="n">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="H5" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="I5" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J5" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="K5" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MLMMJDA14TS</t>
+          <t>MLMMJDA12TXS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3287,81 +3194,435 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Azul Turquesa</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G6" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H6" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="J6" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>MLMMJDA12TXL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Azul Marino</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>16</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MLMMJDA50TXS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>24</v>
+      </c>
+      <c r="G8" t="n">
+        <v>23</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MLMMJDA50TM</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>48</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MLMMJDA66TXS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>24</v>
+      </c>
+      <c r="G10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>25</v>
+      </c>
+      <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MLMMJDA66TL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>24</v>
+      </c>
+      <c r="G11" t="n">
+        <v>22</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="n">
+        <v>20</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MLMMJDA14TXS</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Azul Turquesa</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>24</v>
+      </c>
+      <c r="G12" t="n">
+        <v>20</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" t="n">
+        <v>23</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MLMMJDA14TS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MOTION LOOP MAFE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Azul Turquesa</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>40</v>
+      </c>
+      <c r="G13" t="n">
+        <v>27</v>
+      </c>
+      <c r="H13" t="n">
+        <v>13</v>
+      </c>
+      <c r="I13" t="n">
+        <v>33</v>
+      </c>
+      <c r="J13" t="n">
+        <v>13</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>MLMMJDA14TM</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>MOTION LOOP MAFE</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>DAMA</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Azul Turquesa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>40</v>
-      </c>
-      <c r="G7" t="n">
+      <c r="F14" t="n">
+        <v>40</v>
+      </c>
+      <c r="G14" t="n">
         <v>36</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H14" t="n">
         <v>4</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I14" t="n">
+        <v>32</v>
+      </c>
+      <c r="J14" t="n">
         <v>4</v>
       </c>
-      <c r="J7" t="n">
-        <v>32</v>
-      </c>
-      <c r="K7" t="n">
-        <v>4</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MLCMJCA14TXL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MOTION LOOP CLASICA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CAB</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Azul Turquesa</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>24</v>
+      </c>
+      <c r="G15" t="n">
+        <v>21</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>24</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>